<commit_message>
DACD; extend to 2070
</commit_message>
<xml_diff>
--- a/InputData/geoeng/DACD/Direct Air Capture Data.xlsx
+++ b/InputData/geoeng/DACD/Direct Air Capture Data.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28521"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29530"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Rod\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Olivia Ashmoore\Documents\EPS_Models by Region\eps-mexico\InputData\geoeng\DACD\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1D6638CB-2B61-4B28-88E6-2202EB0466B6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0C9506C3-F44C-4554-919C-87F96A772085}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-90" yWindow="-90" windowWidth="19380" windowHeight="10260" firstSheet="1" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="About" sheetId="1" r:id="rId1"/>
@@ -356,7 +356,7 @@
     <numFmt numFmtId="165" formatCode="0.0%"/>
     <numFmt numFmtId="166" formatCode="0.000E+00"/>
   </numFmts>
-  <fonts count="5">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -431,9 +431,8 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="4">
+  <cellStyleXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="9" fontId="4" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
@@ -445,12 +444,12 @@
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="2"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="11" fontId="0" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
@@ -464,14 +463,13 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="2" applyFont="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="3"/>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="2"/>
   </cellXfs>
-  <cellStyles count="4">
-    <cellStyle name="Hipervínculo" xfId="1" builtinId="8"/>
-    <cellStyle name="Hyperlink" xfId="3" xr:uid="{89AE56F8-F38F-4F16-9D7D-FAE3D047B2C7}"/>
+  <cellStyles count="3">
+    <cellStyle name="Hyperlink" xfId="2" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
-    <cellStyle name="Porcentaje" xfId="2" builtinId="5"/>
+    <cellStyle name="Percent" xfId="1" builtinId="5"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -904,28 +902,28 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:B27"/>
-  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15"/>
+  <sheetFormatPr defaultColWidth="9.1328125" defaultRowHeight="14.75" x14ac:dyDescent="0.75"/>
   <cols>
-    <col min="1" max="1" width="11.140625" customWidth="1"/>
-    <col min="2" max="2" width="47.140625" customWidth="1"/>
+    <col min="1" max="1" width="11.1328125" customWidth="1"/>
+    <col min="2" max="2" width="47.1328125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.75">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="2" spans="1:2">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.75">
       <c r="A2" s="1" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="1:2">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.75">
       <c r="A3" s="1" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="5" spans="1:2">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.75">
       <c r="A5" s="1" t="s">
         <v>3</v>
       </c>
@@ -933,97 +931,97 @@
         <v>4</v>
       </c>
     </row>
-    <row r="6" spans="1:2">
+    <row r="6" spans="1:2" x14ac:dyDescent="0.75">
       <c r="B6" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="7" spans="1:2">
+    <row r="7" spans="1:2" x14ac:dyDescent="0.75">
       <c r="B7" s="6">
         <v>2023</v>
       </c>
     </row>
-    <row r="8" spans="1:2" ht="30">
+    <row r="8" spans="1:2" ht="29.5" x14ac:dyDescent="0.75">
       <c r="B8" s="15" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="9" spans="1:2">
+    <row r="9" spans="1:2" x14ac:dyDescent="0.75">
       <c r="B9" s="19" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="10" spans="1:2">
+    <row r="10" spans="1:2" x14ac:dyDescent="0.75">
       <c r="B10" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="12" spans="1:2">
+    <row r="12" spans="1:2" x14ac:dyDescent="0.75">
       <c r="B12" s="4" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="13" spans="1:2">
+    <row r="13" spans="1:2" x14ac:dyDescent="0.75">
       <c r="B13" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="14" spans="1:2">
+    <row r="14" spans="1:2" x14ac:dyDescent="0.75">
       <c r="B14" s="6">
         <v>2019</v>
       </c>
     </row>
-    <row r="15" spans="1:2">
+    <row r="15" spans="1:2" x14ac:dyDescent="0.75">
       <c r="B15" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="16" spans="1:2">
+    <row r="16" spans="1:2" x14ac:dyDescent="0.75">
       <c r="B16" s="5" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="17" spans="1:2">
+    <row r="17" spans="1:2" x14ac:dyDescent="0.75">
       <c r="B17" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="18" spans="1:2">
+    <row r="18" spans="1:2" x14ac:dyDescent="0.75">
       <c r="B18" s="5" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="19" spans="1:2">
+    <row r="19" spans="1:2" x14ac:dyDescent="0.75">
       <c r="B19" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="21" spans="1:2">
+    <row r="21" spans="1:2" x14ac:dyDescent="0.75">
       <c r="A21" s="1" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="22" spans="1:2">
+    <row r="22" spans="1:2" x14ac:dyDescent="0.75">
       <c r="A22" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="23" spans="1:2">
+    <row r="23" spans="1:2" x14ac:dyDescent="0.75">
       <c r="A23" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="25" spans="1:2">
+    <row r="25" spans="1:2" x14ac:dyDescent="0.75">
       <c r="A25" s="1" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="26" spans="1:2">
+    <row r="26" spans="1:2" x14ac:dyDescent="0.75">
       <c r="A26" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="27" spans="1:2">
+    <row r="27" spans="1:2" x14ac:dyDescent="0.75">
       <c r="A27" t="s">
         <v>21</v>
       </c>
@@ -1042,58 +1040,58 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:H105"/>
-  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15"/>
+  <sheetFormatPr defaultColWidth="9.1328125" defaultRowHeight="14.75" x14ac:dyDescent="0.75"/>
   <cols>
-    <col min="1" max="1" width="33.28515625" customWidth="1"/>
-    <col min="2" max="8" width="11.42578125" customWidth="1"/>
+    <col min="1" max="1" width="33.26953125" customWidth="1"/>
+    <col min="2" max="8" width="11.40625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.75">
       <c r="A1" s="1" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="2" spans="1:7">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.75">
       <c r="A2" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="3" spans="1:7">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.75">
       <c r="A3" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="5" spans="1:7">
+    <row r="5" spans="1:7" x14ac:dyDescent="0.75">
       <c r="A5" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="6" spans="1:7">
+    <row r="6" spans="1:7" x14ac:dyDescent="0.75">
       <c r="A6" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="7" spans="1:7">
+    <row r="7" spans="1:7" x14ac:dyDescent="0.75">
       <c r="A7" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="8" spans="1:7">
+    <row r="8" spans="1:7" x14ac:dyDescent="0.75">
       <c r="A8" t="s">
         <v>28</v>
       </c>
     </row>
-    <row r="9" spans="1:7">
+    <row r="9" spans="1:7" x14ac:dyDescent="0.75">
       <c r="A9" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="11" spans="1:7">
+    <row r="11" spans="1:7" x14ac:dyDescent="0.75">
       <c r="A11" s="1" t="s">
         <v>30</v>
       </c>
     </row>
-    <row r="12" spans="1:7">
+    <row r="12" spans="1:7" x14ac:dyDescent="0.75">
       <c r="A12" s="13" t="s">
         <v>31</v>
       </c>
@@ -1104,7 +1102,7 @@
       <c r="F12" s="14"/>
       <c r="G12" s="14"/>
     </row>
-    <row r="13" spans="1:7">
+    <row r="13" spans="1:7" x14ac:dyDescent="0.75">
       <c r="A13" s="2" t="s">
         <v>32</v>
       </c>
@@ -1115,7 +1113,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="14" spans="1:7">
+    <row r="14" spans="1:7" x14ac:dyDescent="0.75">
       <c r="A14" s="1" t="s">
         <v>35</v>
       </c>
@@ -1126,7 +1124,7 @@
         <v>350</v>
       </c>
     </row>
-    <row r="15" spans="1:7">
+    <row r="15" spans="1:7" x14ac:dyDescent="0.75">
       <c r="A15" s="1" t="s">
         <v>36</v>
       </c>
@@ -1137,7 +1135,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="16" spans="1:7">
+    <row r="16" spans="1:7" x14ac:dyDescent="0.75">
       <c r="A16" s="1" t="s">
         <v>37</v>
       </c>
@@ -1148,12 +1146,12 @@
         <v>50</v>
       </c>
     </row>
-    <row r="18" spans="1:4">
+    <row r="18" spans="1:4" x14ac:dyDescent="0.75">
       <c r="A18" s="1" t="s">
         <v>38</v>
       </c>
     </row>
-    <row r="19" spans="1:4">
+    <row r="19" spans="1:4" x14ac:dyDescent="0.75">
       <c r="A19" s="2" t="s">
         <v>39</v>
       </c>
@@ -1164,7 +1162,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="20" spans="1:4">
+    <row r="20" spans="1:4" x14ac:dyDescent="0.75">
       <c r="A20" s="1" t="s">
         <v>35</v>
       </c>
@@ -1175,7 +1173,7 @@
         <v>1.1000000000000001</v>
       </c>
     </row>
-    <row r="21" spans="1:4">
+    <row r="21" spans="1:4" x14ac:dyDescent="0.75">
       <c r="A21" s="1" t="s">
         <v>36</v>
       </c>
@@ -1186,17 +1184,17 @@
         <v>0.6</v>
       </c>
     </row>
-    <row r="22" spans="1:4">
+    <row r="22" spans="1:4" x14ac:dyDescent="0.75">
       <c r="A22" s="1" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="24" spans="1:4">
+    <row r="24" spans="1:4" x14ac:dyDescent="0.75">
       <c r="A24" s="1" t="s">
         <v>40</v>
       </c>
     </row>
-    <row r="25" spans="1:4">
+    <row r="25" spans="1:4" x14ac:dyDescent="0.75">
       <c r="A25" s="2" t="s">
         <v>39</v>
       </c>
@@ -1207,7 +1205,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="26" spans="1:4">
+    <row r="26" spans="1:4" x14ac:dyDescent="0.75">
       <c r="A26" s="1" t="s">
         <v>35</v>
       </c>
@@ -1218,7 +1216,7 @@
         <v>7.2</v>
       </c>
     </row>
-    <row r="27" spans="1:4">
+    <row r="27" spans="1:4" x14ac:dyDescent="0.75">
       <c r="A27" s="1" t="s">
         <v>36</v>
       </c>
@@ -1229,15 +1227,15 @@
         <v>4.4000000000000004</v>
       </c>
     </row>
-    <row r="28" spans="1:4">
+    <row r="28" spans="1:4" x14ac:dyDescent="0.75">
       <c r="A28" s="1" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="29" spans="1:4">
+    <row r="29" spans="1:4" x14ac:dyDescent="0.75">
       <c r="A29" s="1"/>
     </row>
-    <row r="30" spans="1:4" ht="30">
+    <row r="30" spans="1:4" ht="29.5" x14ac:dyDescent="0.75">
       <c r="A30" s="17" t="s">
         <v>41</v>
       </c>
@@ -1248,15 +1246,15 @@
         <v>42</v>
       </c>
     </row>
-    <row r="31" spans="1:4">
+    <row r="31" spans="1:4" x14ac:dyDescent="0.75">
       <c r="A31" s="1"/>
     </row>
-    <row r="32" spans="1:4">
+    <row r="32" spans="1:4" x14ac:dyDescent="0.75">
       <c r="A32" s="1" t="s">
         <v>43</v>
       </c>
     </row>
-    <row r="33" spans="1:3">
+    <row r="33" spans="1:3" x14ac:dyDescent="0.75">
       <c r="A33" s="2" t="s">
         <v>39</v>
       </c>
@@ -1267,7 +1265,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="34" spans="1:3">
+    <row r="34" spans="1:3" x14ac:dyDescent="0.75">
       <c r="A34" s="1" t="s">
         <v>35</v>
       </c>
@@ -1280,7 +1278,7 @@
         <v>2.3759999999999999</v>
       </c>
     </row>
-    <row r="35" spans="1:3">
+    <row r="35" spans="1:3" x14ac:dyDescent="0.75">
       <c r="A35" s="1" t="s">
         <v>36</v>
       </c>
@@ -1293,27 +1291,27 @@
         <v>1.452</v>
       </c>
     </row>
-    <row r="37" spans="1:3">
+    <row r="37" spans="1:3" x14ac:dyDescent="0.75">
       <c r="A37" s="1" t="s">
         <v>44</v>
       </c>
     </row>
-    <row r="38" spans="1:3">
+    <row r="38" spans="1:3" x14ac:dyDescent="0.75">
       <c r="A38" t="s">
         <v>45</v>
       </c>
     </row>
-    <row r="39" spans="1:3">
+    <row r="39" spans="1:3" x14ac:dyDescent="0.75">
       <c r="A39" t="s">
         <v>46</v>
       </c>
     </row>
-    <row r="40" spans="1:3">
+    <row r="40" spans="1:3" x14ac:dyDescent="0.75">
       <c r="A40" t="s">
         <v>47</v>
       </c>
     </row>
-    <row r="62" spans="1:8">
+    <row r="62" spans="1:8" x14ac:dyDescent="0.75">
       <c r="A62" s="4" t="s">
         <v>48</v>
       </c>
@@ -1325,27 +1323,27 @@
       <c r="G62" s="9"/>
       <c r="H62" s="9"/>
     </row>
-    <row r="63" spans="1:8">
+    <row r="63" spans="1:8" x14ac:dyDescent="0.75">
       <c r="A63" t="s">
         <v>49</v>
       </c>
     </row>
-    <row r="64" spans="1:8">
+    <row r="64" spans="1:8" x14ac:dyDescent="0.75">
       <c r="A64" t="s">
         <v>50</v>
       </c>
     </row>
-    <row r="65" spans="1:8">
+    <row r="65" spans="1:8" x14ac:dyDescent="0.75">
       <c r="A65" t="s">
         <v>51</v>
       </c>
     </row>
-    <row r="66" spans="1:8">
+    <row r="66" spans="1:8" x14ac:dyDescent="0.75">
       <c r="A66" t="s">
         <v>52</v>
       </c>
     </row>
-    <row r="68" spans="1:8">
+    <row r="68" spans="1:8" x14ac:dyDescent="0.75">
       <c r="B68">
         <v>2045</v>
       </c>
@@ -1368,7 +1366,7 @@
         <v>2100</v>
       </c>
     </row>
-    <row r="69" spans="1:8">
+    <row r="69" spans="1:8" x14ac:dyDescent="0.75">
       <c r="A69" t="s">
         <v>53</v>
       </c>
@@ -1394,7 +1392,7 @@
         <v>379</v>
       </c>
     </row>
-    <row r="70" spans="1:8">
+    <row r="70" spans="1:8" x14ac:dyDescent="0.75">
       <c r="A70" t="s">
         <v>54</v>
       </c>
@@ -1420,7 +1418,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="72" spans="1:8">
+    <row r="72" spans="1:8" x14ac:dyDescent="0.75">
       <c r="A72" t="s">
         <v>55</v>
       </c>
@@ -1428,7 +1426,7 @@
         <v>420</v>
       </c>
     </row>
-    <row r="74" spans="1:8">
+    <row r="74" spans="1:8" x14ac:dyDescent="0.75">
       <c r="B74">
         <v>2045</v>
       </c>
@@ -1451,7 +1449,7 @@
         <v>2100</v>
       </c>
     </row>
-    <row r="75" spans="1:8">
+    <row r="75" spans="1:8" x14ac:dyDescent="0.75">
       <c r="A75" t="s">
         <v>56</v>
       </c>
@@ -1484,7 +1482,7 @@
         <v>27.071428571428573</v>
       </c>
     </row>
-    <row r="76" spans="1:8">
+    <row r="76" spans="1:8" x14ac:dyDescent="0.75">
       <c r="A76" t="s">
         <v>57</v>
       </c>
@@ -1517,27 +1515,27 @@
         <v>2.8571428571428568</v>
       </c>
     </row>
-    <row r="78" spans="1:8">
+    <row r="78" spans="1:8" x14ac:dyDescent="0.75">
       <c r="A78" s="1" t="s">
         <v>58</v>
       </c>
     </row>
-    <row r="79" spans="1:8">
+    <row r="79" spans="1:8" x14ac:dyDescent="0.75">
       <c r="A79" t="s">
         <v>59</v>
       </c>
     </row>
-    <row r="80" spans="1:8">
+    <row r="80" spans="1:8" x14ac:dyDescent="0.75">
       <c r="A80" t="s">
         <v>60</v>
       </c>
     </row>
-    <row r="81" spans="1:8">
+    <row r="81" spans="1:8" x14ac:dyDescent="0.75">
       <c r="A81" t="s">
         <v>61</v>
       </c>
     </row>
-    <row r="83" spans="1:8">
+    <row r="83" spans="1:8" x14ac:dyDescent="0.75">
       <c r="A83" t="s">
         <v>62</v>
       </c>
@@ -1551,7 +1549,7 @@
         <v>2017</v>
       </c>
     </row>
-    <row r="84" spans="1:8">
+    <row r="84" spans="1:8" x14ac:dyDescent="0.75">
       <c r="A84" t="s">
         <v>64</v>
       </c>
@@ -1565,7 +1563,7 @@
         <v>2017</v>
       </c>
     </row>
-    <row r="85" spans="1:8">
+    <row r="85" spans="1:8" x14ac:dyDescent="0.75">
       <c r="A85" t="s">
         <v>66</v>
       </c>
@@ -1574,7 +1572,7 @@
         <v>0.24237500000000001</v>
       </c>
     </row>
-    <row r="87" spans="1:8">
+    <row r="87" spans="1:8" x14ac:dyDescent="0.75">
       <c r="A87" s="4" t="s">
         <v>67</v>
       </c>
@@ -1586,7 +1584,7 @@
       <c r="G87" s="9"/>
       <c r="H87" s="9"/>
     </row>
-    <row r="88" spans="1:8">
+    <row r="88" spans="1:8" x14ac:dyDescent="0.75">
       <c r="B88">
         <v>2045</v>
       </c>
@@ -1609,7 +1607,7 @@
         <v>2100</v>
       </c>
     </row>
-    <row r="89" spans="1:8">
+    <row r="89" spans="1:8" x14ac:dyDescent="0.75">
       <c r="A89" t="s">
         <v>56</v>
       </c>
@@ -1642,7 +1640,7 @@
         <v>6.5614375000000003</v>
       </c>
     </row>
-    <row r="90" spans="1:8">
+    <row r="90" spans="1:8" x14ac:dyDescent="0.75">
       <c r="A90" t="s">
         <v>57</v>
       </c>
@@ -1675,12 +1673,12 @@
         <v>0.69249999999999989</v>
       </c>
     </row>
-    <row r="92" spans="1:8">
+    <row r="92" spans="1:8" x14ac:dyDescent="0.75">
       <c r="A92" t="s">
         <v>68</v>
       </c>
     </row>
-    <row r="93" spans="1:8">
+    <row r="93" spans="1:8" x14ac:dyDescent="0.75">
       <c r="B93">
         <v>2045</v>
       </c>
@@ -1703,7 +1701,7 @@
         <v>2100</v>
       </c>
     </row>
-    <row r="94" spans="1:8">
+    <row r="94" spans="1:8" x14ac:dyDescent="0.75">
       <c r="A94" t="s">
         <v>69</v>
       </c>
@@ -1736,7 +1734,7 @@
         <v>6561437500</v>
       </c>
     </row>
-    <row r="95" spans="1:8">
+    <row r="95" spans="1:8" x14ac:dyDescent="0.75">
       <c r="A95" t="s">
         <v>70</v>
       </c>
@@ -1769,32 +1767,32 @@
         <v>692499999.99999988</v>
       </c>
     </row>
-    <row r="97" spans="1:2">
+    <row r="97" spans="1:2" x14ac:dyDescent="0.75">
       <c r="A97" s="4" t="s">
         <v>71</v>
       </c>
     </row>
-    <row r="98" spans="1:2">
+    <row r="98" spans="1:2" x14ac:dyDescent="0.75">
       <c r="A98" t="s">
         <v>72</v>
       </c>
     </row>
-    <row r="99" spans="1:2">
+    <row r="99" spans="1:2" x14ac:dyDescent="0.75">
       <c r="A99" t="s">
         <v>73</v>
       </c>
     </row>
-    <row r="100" spans="1:2">
+    <row r="100" spans="1:2" x14ac:dyDescent="0.75">
       <c r="A100" t="s">
         <v>74</v>
       </c>
     </row>
-    <row r="101" spans="1:2">
+    <row r="101" spans="1:2" x14ac:dyDescent="0.75">
       <c r="A101" t="s">
         <v>75</v>
       </c>
     </row>
-    <row r="103" spans="1:2">
+    <row r="103" spans="1:2" x14ac:dyDescent="0.75">
       <c r="A103" t="s">
         <v>76</v>
       </c>
@@ -1802,7 +1800,7 @@
         <v>947086</v>
       </c>
     </row>
-    <row r="105" spans="1:2">
+    <row r="105" spans="1:2" x14ac:dyDescent="0.75">
       <c r="A105" t="s">
         <v>77</v>
       </c>
@@ -1817,9 +1815,9 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{89E4CEC2-71D6-45C4-AD10-306F02D88CEB}">
   <dimension ref="A1:B1"/>
-  <sheetFormatPr defaultColWidth="11.42578125" defaultRowHeight="15"/>
+  <sheetFormatPr defaultColWidth="11.40625" defaultRowHeight="14.75" x14ac:dyDescent="0.75"/>
   <sheetData>
-    <row r="1" spans="1:2" ht="30">
+    <row r="1" spans="1:2" ht="29.5" x14ac:dyDescent="0.75">
       <c r="A1" s="15" t="s">
         <v>78</v>
       </c>
@@ -1839,19 +1837,19 @@
     <tabColor theme="8" tint="-0.249977111117893"/>
   </sheetPr>
   <dimension ref="A1:BC2"/>
-  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15"/>
+  <sheetFormatPr defaultColWidth="9.1328125" defaultRowHeight="14.75" x14ac:dyDescent="0.75"/>
   <cols>
-    <col min="1" max="1" width="19.85546875" customWidth="1"/>
-    <col min="2" max="2" width="9.140625" customWidth="1"/>
-    <col min="3" max="9" width="9.42578125" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="10.28515625" bestFit="1" customWidth="1"/>
-    <col min="11" max="24" width="9.42578125" bestFit="1" customWidth="1"/>
-    <col min="25" max="25" width="10.85546875" bestFit="1" customWidth="1"/>
-    <col min="26" max="35" width="9.42578125" bestFit="1" customWidth="1"/>
-    <col min="36" max="36" width="9.5703125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="19.86328125" customWidth="1"/>
+    <col min="2" max="2" width="9.1328125" customWidth="1"/>
+    <col min="3" max="9" width="9.40625" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="10.26953125" bestFit="1" customWidth="1"/>
+    <col min="11" max="24" width="9.40625" bestFit="1" customWidth="1"/>
+    <col min="25" max="25" width="10.86328125" bestFit="1" customWidth="1"/>
+    <col min="26" max="35" width="9.40625" bestFit="1" customWidth="1"/>
+    <col min="36" max="36" width="9.54296875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:55">
+    <row r="1" spans="1:55" x14ac:dyDescent="0.75">
       <c r="A1" s="2" t="s">
         <v>79</v>
       </c>
@@ -2018,7 +2016,7 @@
         <v>2070</v>
       </c>
     </row>
-    <row r="2" spans="1:55">
+    <row r="2" spans="1:55" x14ac:dyDescent="0.75">
       <c r="A2" t="s">
         <v>80</v>
       </c>
@@ -2242,14 +2240,14 @@
   <sheetPr>
     <tabColor theme="8" tint="-0.249977111117893"/>
   </sheetPr>
-  <dimension ref="A1:AI11"/>
-  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15"/>
+  <dimension ref="A1:BC11"/>
+  <sheetFormatPr defaultColWidth="9.1328125" defaultRowHeight="14.75" x14ac:dyDescent="0.75"/>
   <cols>
-    <col min="1" max="1" width="24.7109375" customWidth="1"/>
-    <col min="2" max="2" width="9.140625" customWidth="1"/>
+    <col min="1" max="1" width="24.7265625" customWidth="1"/>
+    <col min="2" max="2" width="9.1328125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:35">
+    <row r="1" spans="1:55" x14ac:dyDescent="0.75">
       <c r="A1" s="2" t="s">
         <v>81</v>
       </c>
@@ -2355,8 +2353,68 @@
       <c r="AI1">
         <v>2050</v>
       </c>
-    </row>
-    <row r="2" spans="1:35">
+      <c r="AJ1">
+        <v>2051</v>
+      </c>
+      <c r="AK1">
+        <v>2052</v>
+      </c>
+      <c r="AL1">
+        <v>2053</v>
+      </c>
+      <c r="AM1">
+        <v>2054</v>
+      </c>
+      <c r="AN1">
+        <v>2055</v>
+      </c>
+      <c r="AO1">
+        <v>2056</v>
+      </c>
+      <c r="AP1">
+        <v>2057</v>
+      </c>
+      <c r="AQ1">
+        <v>2058</v>
+      </c>
+      <c r="AR1">
+        <v>2059</v>
+      </c>
+      <c r="AS1">
+        <v>2060</v>
+      </c>
+      <c r="AT1">
+        <v>2061</v>
+      </c>
+      <c r="AU1">
+        <v>2062</v>
+      </c>
+      <c r="AV1">
+        <v>2063</v>
+      </c>
+      <c r="AW1">
+        <v>2064</v>
+      </c>
+      <c r="AX1">
+        <v>2065</v>
+      </c>
+      <c r="AY1">
+        <v>2066</v>
+      </c>
+      <c r="AZ1">
+        <v>2067</v>
+      </c>
+      <c r="BA1">
+        <v>2068</v>
+      </c>
+      <c r="BB1">
+        <v>2069</v>
+      </c>
+      <c r="BC1">
+        <v>2070</v>
+      </c>
+    </row>
+    <row r="2" spans="1:55" x14ac:dyDescent="0.75">
       <c r="A2" t="s">
         <v>82</v>
       </c>
@@ -2496,8 +2554,88 @@
         <f t="shared" si="0"/>
         <v>4236315.6780000003</v>
       </c>
-    </row>
-    <row r="3" spans="1:35">
+      <c r="AJ2" s="12">
+        <f t="shared" ref="AJ2:AZ11" si="1">$B2</f>
+        <v>4236315.6780000003</v>
+      </c>
+      <c r="AK2" s="12">
+        <f t="shared" si="1"/>
+        <v>4236315.6780000003</v>
+      </c>
+      <c r="AL2" s="12">
+        <f t="shared" si="1"/>
+        <v>4236315.6780000003</v>
+      </c>
+      <c r="AM2" s="12">
+        <f t="shared" si="1"/>
+        <v>4236315.6780000003</v>
+      </c>
+      <c r="AN2" s="12">
+        <f t="shared" si="1"/>
+        <v>4236315.6780000003</v>
+      </c>
+      <c r="AO2" s="12">
+        <f t="shared" si="1"/>
+        <v>4236315.6780000003</v>
+      </c>
+      <c r="AP2" s="12">
+        <f t="shared" si="1"/>
+        <v>4236315.6780000003</v>
+      </c>
+      <c r="AQ2" s="12">
+        <f t="shared" si="1"/>
+        <v>4236315.6780000003</v>
+      </c>
+      <c r="AR2" s="12">
+        <f t="shared" si="1"/>
+        <v>4236315.6780000003</v>
+      </c>
+      <c r="AS2" s="12">
+        <f t="shared" si="1"/>
+        <v>4236315.6780000003</v>
+      </c>
+      <c r="AT2" s="12">
+        <f t="shared" si="1"/>
+        <v>4236315.6780000003</v>
+      </c>
+      <c r="AU2" s="12">
+        <f t="shared" si="1"/>
+        <v>4236315.6780000003</v>
+      </c>
+      <c r="AV2" s="12">
+        <f t="shared" si="1"/>
+        <v>4236315.6780000003</v>
+      </c>
+      <c r="AW2" s="12">
+        <f t="shared" si="1"/>
+        <v>4236315.6780000003</v>
+      </c>
+      <c r="AX2" s="12">
+        <f t="shared" si="1"/>
+        <v>4236315.6780000003</v>
+      </c>
+      <c r="AY2" s="12">
+        <f t="shared" si="1"/>
+        <v>4236315.6780000003</v>
+      </c>
+      <c r="AZ2" s="12">
+        <f t="shared" si="1"/>
+        <v>4236315.6780000003</v>
+      </c>
+      <c r="BA2" s="12">
+        <f t="shared" ref="BA2:BC11" si="2">$B2</f>
+        <v>4236315.6780000003</v>
+      </c>
+      <c r="BB2" s="12">
+        <f t="shared" si="2"/>
+        <v>4236315.6780000003</v>
+      </c>
+      <c r="BC2" s="12">
+        <f t="shared" si="2"/>
+        <v>4236315.6780000003</v>
+      </c>
+    </row>
+    <row r="3" spans="1:55" x14ac:dyDescent="0.75">
       <c r="A3" t="s">
         <v>83</v>
       </c>
@@ -2505,67 +2643,67 @@
         <v>0</v>
       </c>
       <c r="C3" s="12">
-        <f t="shared" ref="C3:R11" si="1">$B3</f>
+        <f t="shared" ref="C3:R11" si="3">$B3</f>
         <v>0</v>
       </c>
       <c r="D3" s="12">
-        <f t="shared" si="1"/>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="E3" s="12">
-        <f t="shared" si="1"/>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="F3" s="12">
-        <f t="shared" si="1"/>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="G3" s="12">
-        <f t="shared" si="1"/>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="H3" s="12">
-        <f t="shared" si="1"/>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="I3" s="12">
-        <f t="shared" si="1"/>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="J3" s="12">
-        <f t="shared" si="1"/>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="K3" s="12">
-        <f t="shared" si="1"/>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="L3" s="12">
-        <f t="shared" si="1"/>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="M3" s="12">
-        <f t="shared" si="1"/>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="N3" s="12">
-        <f t="shared" si="1"/>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="O3" s="12">
-        <f t="shared" si="1"/>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="P3" s="12">
-        <f t="shared" si="1"/>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="Q3" s="12">
-        <f t="shared" si="1"/>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="R3" s="12">
-        <f t="shared" si="1"/>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="S3" s="12">
@@ -2636,8 +2774,88 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-    </row>
-    <row r="4" spans="1:35">
+      <c r="AJ3" s="12">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="AK3" s="12">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="AL3" s="12">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="AM3" s="12">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="AN3" s="12">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="AO3" s="12">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="AP3" s="12">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="AQ3" s="12">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="AR3" s="12">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="AS3" s="12">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="AT3" s="12">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="AU3" s="12">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="AV3" s="12">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="AW3" s="12">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="AX3" s="12">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="AY3" s="12">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="AZ3" s="12">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="BA3" s="12">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="BB3" s="12">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="BC3" s="12">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4" spans="1:55" x14ac:dyDescent="0.75">
       <c r="A4" t="s">
         <v>84</v>
       </c>
@@ -2645,7 +2863,7 @@
         <v>0</v>
       </c>
       <c r="C4" s="12">
-        <f t="shared" si="1"/>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="D4" s="12">
@@ -2776,8 +2994,88 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-    </row>
-    <row r="5" spans="1:35">
+      <c r="AJ4" s="12">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="AK4" s="12">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="AL4" s="12">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="AM4" s="12">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="AN4" s="12">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="AO4" s="12">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="AP4" s="12">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="AQ4" s="12">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="AR4" s="12">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="AS4" s="12">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="AT4" s="12">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="AU4" s="12">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="AV4" s="12">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="AW4" s="12">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="AX4" s="12">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="AY4" s="12">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="AZ4" s="12">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="BA4" s="12">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="BB4" s="12">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="BC4" s="12">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5" spans="1:55" x14ac:dyDescent="0.75">
       <c r="A5" t="s">
         <v>85</v>
       </c>
@@ -2785,7 +3083,7 @@
         <v>0</v>
       </c>
       <c r="C5" s="12">
-        <f t="shared" si="1"/>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="D5" s="12">
@@ -2916,8 +3214,88 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-    </row>
-    <row r="6" spans="1:35">
+      <c r="AJ5" s="12">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="AK5" s="12">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="AL5" s="12">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="AM5" s="12">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="AN5" s="12">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="AO5" s="12">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="AP5" s="12">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="AQ5" s="12">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="AR5" s="12">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="AS5" s="12">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="AT5" s="12">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="AU5" s="12">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="AV5" s="12">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="AW5" s="12">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="AX5" s="12">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="AY5" s="12">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="AZ5" s="12">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="BA5" s="12">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="BB5" s="12">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="BC5" s="12">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6" spans="1:55" x14ac:dyDescent="0.75">
       <c r="A6" t="s">
         <v>86</v>
       </c>
@@ -2925,7 +3303,7 @@
         <v>0</v>
       </c>
       <c r="C6" s="12">
-        <f t="shared" si="1"/>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="D6" s="12">
@@ -3056,8 +3434,88 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-    </row>
-    <row r="7" spans="1:35">
+      <c r="AJ6" s="12">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="AK6" s="12">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="AL6" s="12">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="AM6" s="12">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="AN6" s="12">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="AO6" s="12">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="AP6" s="12">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="AQ6" s="12">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="AR6" s="12">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="AS6" s="12">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="AT6" s="12">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="AU6" s="12">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="AV6" s="12">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="AW6" s="12">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="AX6" s="12">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="AY6" s="12">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="AZ6" s="12">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="BA6" s="12">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="BB6" s="12">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="BC6" s="12">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7" spans="1:55" x14ac:dyDescent="0.75">
       <c r="A7" t="s">
         <v>87</v>
       </c>
@@ -3065,7 +3523,7 @@
         <v>0</v>
       </c>
       <c r="C7" s="12">
-        <f t="shared" si="1"/>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="D7" s="12">
@@ -3196,8 +3654,88 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-    </row>
-    <row r="8" spans="1:35">
+      <c r="AJ7" s="12">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="AK7" s="12">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="AL7" s="12">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="AM7" s="12">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="AN7" s="12">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="AO7" s="12">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="AP7" s="12">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="AQ7" s="12">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="AR7" s="12">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="AS7" s="12">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="AT7" s="12">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="AU7" s="12">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="AV7" s="12">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="AW7" s="12">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="AX7" s="12">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="AY7" s="12">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="AZ7" s="12">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="BA7" s="12">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="BB7" s="12">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="BC7" s="12">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8" spans="1:55" x14ac:dyDescent="0.75">
       <c r="A8" t="s">
         <v>88</v>
       </c>
@@ -3205,7 +3743,7 @@
         <v>0</v>
       </c>
       <c r="C8" s="12">
-        <f t="shared" si="1"/>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="D8" s="12">
@@ -3336,8 +3874,88 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-    </row>
-    <row r="9" spans="1:35">
+      <c r="AJ8" s="12">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="AK8" s="12">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="AL8" s="12">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="AM8" s="12">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="AN8" s="12">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="AO8" s="12">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="AP8" s="12">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="AQ8" s="12">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="AR8" s="12">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="AS8" s="12">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="AT8" s="12">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="AU8" s="12">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="AV8" s="12">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="AW8" s="12">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="AX8" s="12">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="AY8" s="12">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="AZ8" s="12">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="BA8" s="12">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="BB8" s="12">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="BC8" s="12">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9" spans="1:55" x14ac:dyDescent="0.75">
       <c r="A9" t="s">
         <v>89</v>
       </c>
@@ -3345,7 +3963,7 @@
         <v>0</v>
       </c>
       <c r="C9" s="12">
-        <f t="shared" si="1"/>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="D9" s="12">
@@ -3476,8 +4094,88 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-    </row>
-    <row r="10" spans="1:35">
+      <c r="AJ9" s="12">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="AK9" s="12">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="AL9" s="12">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="AM9" s="12">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="AN9" s="12">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="AO9" s="12">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="AP9" s="12">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="AQ9" s="12">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="AR9" s="12">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="AS9" s="12">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="AT9" s="12">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="AU9" s="12">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="AV9" s="12">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="AW9" s="12">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="AX9" s="12">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="AY9" s="12">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="AZ9" s="12">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="BA9" s="12">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="BB9" s="12">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="BC9" s="12">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="10" spans="1:55" x14ac:dyDescent="0.75">
       <c r="A10" t="s">
         <v>90</v>
       </c>
@@ -3485,7 +4183,7 @@
         <v>0</v>
       </c>
       <c r="C10" s="12">
-        <f t="shared" si="1"/>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="D10" s="12">
@@ -3545,79 +4243,159 @@
         <v>0</v>
       </c>
       <c r="R10" s="12">
-        <f t="shared" ref="D10:AI11" si="2">$B10</f>
+        <f t="shared" ref="D10:AJ11" si="4">$B10</f>
         <v>0</v>
       </c>
       <c r="S10" s="12">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="T10" s="12">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="U10" s="12">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="V10" s="12">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="W10" s="12">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="X10" s="12">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="Y10" s="12">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="Z10" s="12">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="AA10" s="12">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="AB10" s="12">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="AC10" s="12">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="AD10" s="12">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="AE10" s="12">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="AF10" s="12">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="AG10" s="12">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="AH10" s="12">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="AI10" s="12">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="AJ10" s="12">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="AK10" s="12">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="AL10" s="12">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="AM10" s="12">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="AN10" s="12">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="AO10" s="12">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="AP10" s="12">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="AQ10" s="12">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="AR10" s="12">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="AS10" s="12">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="AT10" s="12">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="AU10" s="12">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="AV10" s="12">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="AW10" s="12">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="AX10" s="12">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="AY10" s="12">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="AZ10" s="12">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="BA10" s="12">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-      <c r="T10" s="12">
+      <c r="BB10" s="12">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-      <c r="U10" s="12">
+      <c r="BC10" s="12">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-      <c r="V10" s="12">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="W10" s="12">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="X10" s="12">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="Y10" s="12">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="Z10" s="12">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="AA10" s="12">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="AB10" s="12">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="AC10" s="12">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="AD10" s="12">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="AE10" s="12">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="AF10" s="12">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="AG10" s="12">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="AH10" s="12">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="AI10" s="12">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="11" spans="1:35">
+    </row>
+    <row r="11" spans="1:55" x14ac:dyDescent="0.75">
       <c r="A11" t="s">
         <v>91</v>
       </c>
@@ -3625,134 +4403,214 @@
         <v>0</v>
       </c>
       <c r="C11" s="12">
-        <f t="shared" si="1"/>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="D11" s="12">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="E11" s="12">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="F11" s="12">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="G11" s="12">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="H11" s="12">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="I11" s="12">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="J11" s="12">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="K11" s="12">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="L11" s="12">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="M11" s="12">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="N11" s="12">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="O11" s="12">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="P11" s="12">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="Q11" s="12">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="R11" s="12">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="S11" s="12">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="T11" s="12">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="U11" s="12">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="V11" s="12">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="W11" s="12">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="X11" s="12">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="Y11" s="12">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="Z11" s="12">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="AA11" s="12">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="AB11" s="12">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="AC11" s="12">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="AD11" s="12">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="AE11" s="12">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="AF11" s="12">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="AG11" s="12">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="AH11" s="12">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="AI11" s="12">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="AJ11" s="12">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="AK11" s="12">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="AL11" s="12">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="AM11" s="12">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="AN11" s="12">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="AO11" s="12">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="AP11" s="12">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="AQ11" s="12">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="AR11" s="12">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="AS11" s="12">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="AT11" s="12">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="AU11" s="12">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="AV11" s="12">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="AW11" s="12">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="AX11" s="12">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="AY11" s="12">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="AZ11" s="12">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="BA11" s="12">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-      <c r="E11" s="12">
+      <c r="BB11" s="12">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-      <c r="F11" s="12">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="G11" s="12">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="H11" s="12">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="I11" s="12">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="J11" s="12">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="K11" s="12">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="L11" s="12">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="M11" s="12">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="N11" s="12">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="O11" s="12">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="P11" s="12">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="Q11" s="12">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="R11" s="12">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="S11" s="12">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="T11" s="12">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="U11" s="12">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="V11" s="12">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="W11" s="12">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="X11" s="12">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="Y11" s="12">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="Z11" s="12">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="AA11" s="12">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="AB11" s="12">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="AC11" s="12">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="AD11" s="12">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="AE11" s="12">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="AF11" s="12">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="AG11" s="12">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="AH11" s="12">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="AI11" s="12">
+      <c r="BC11" s="12">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
@@ -3767,14 +4625,14 @@
   <sheetPr>
     <tabColor theme="8" tint="-0.249977111117893"/>
   </sheetPr>
-  <dimension ref="A1:AI2"/>
-  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15"/>
+  <dimension ref="A1:BC2"/>
+  <sheetFormatPr defaultColWidth="9.1328125" defaultRowHeight="14.75" x14ac:dyDescent="0.75"/>
   <cols>
-    <col min="1" max="1" width="24.7109375" customWidth="1"/>
-    <col min="2" max="2" width="9.140625" customWidth="1"/>
+    <col min="1" max="1" width="24.7265625" customWidth="1"/>
+    <col min="2" max="2" width="9.1328125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:35">
+    <row r="1" spans="1:55" x14ac:dyDescent="0.75">
       <c r="A1" s="2" t="s">
         <v>92</v>
       </c>
@@ -3880,8 +4738,68 @@
       <c r="AI1">
         <v>2050</v>
       </c>
-    </row>
-    <row r="2" spans="1:35">
+      <c r="AJ1">
+        <v>2051</v>
+      </c>
+      <c r="AK1">
+        <v>2052</v>
+      </c>
+      <c r="AL1">
+        <v>2053</v>
+      </c>
+      <c r="AM1">
+        <v>2054</v>
+      </c>
+      <c r="AN1">
+        <v>2055</v>
+      </c>
+      <c r="AO1">
+        <v>2056</v>
+      </c>
+      <c r="AP1">
+        <v>2057</v>
+      </c>
+      <c r="AQ1">
+        <v>2058</v>
+      </c>
+      <c r="AR1">
+        <v>2059</v>
+      </c>
+      <c r="AS1">
+        <v>2060</v>
+      </c>
+      <c r="AT1">
+        <v>2061</v>
+      </c>
+      <c r="AU1">
+        <v>2062</v>
+      </c>
+      <c r="AV1">
+        <v>2063</v>
+      </c>
+      <c r="AW1">
+        <v>2064</v>
+      </c>
+      <c r="AX1">
+        <v>2065</v>
+      </c>
+      <c r="AY1">
+        <v>2066</v>
+      </c>
+      <c r="AZ1">
+        <v>2067</v>
+      </c>
+      <c r="BA1">
+        <v>2068</v>
+      </c>
+      <c r="BB1">
+        <v>2069</v>
+      </c>
+      <c r="BC1">
+        <v>2070</v>
+      </c>
+    </row>
+    <row r="2" spans="1:55" x14ac:dyDescent="0.75">
       <c r="A2" t="s">
         <v>93</v>
       </c>
@@ -3894,7 +4812,7 @@
         <v>300</v>
       </c>
       <c r="D2" s="12">
-        <f t="shared" ref="D2:AI2" si="0">$B2</f>
+        <f t="shared" ref="D2:BC2" si="0">$B2</f>
         <v>300</v>
       </c>
       <c r="E2" s="12">
@@ -4018,6 +4936,86 @@
         <v>300</v>
       </c>
       <c r="AI2" s="12">
+        <f t="shared" si="0"/>
+        <v>300</v>
+      </c>
+      <c r="AJ2" s="12">
+        <f t="shared" si="0"/>
+        <v>300</v>
+      </c>
+      <c r="AK2" s="12">
+        <f t="shared" si="0"/>
+        <v>300</v>
+      </c>
+      <c r="AL2" s="12">
+        <f t="shared" si="0"/>
+        <v>300</v>
+      </c>
+      <c r="AM2" s="12">
+        <f t="shared" si="0"/>
+        <v>300</v>
+      </c>
+      <c r="AN2" s="12">
+        <f t="shared" si="0"/>
+        <v>300</v>
+      </c>
+      <c r="AO2" s="12">
+        <f t="shared" si="0"/>
+        <v>300</v>
+      </c>
+      <c r="AP2" s="12">
+        <f t="shared" si="0"/>
+        <v>300</v>
+      </c>
+      <c r="AQ2" s="12">
+        <f t="shared" si="0"/>
+        <v>300</v>
+      </c>
+      <c r="AR2" s="12">
+        <f t="shared" si="0"/>
+        <v>300</v>
+      </c>
+      <c r="AS2" s="12">
+        <f t="shared" si="0"/>
+        <v>300</v>
+      </c>
+      <c r="AT2" s="12">
+        <f t="shared" si="0"/>
+        <v>300</v>
+      </c>
+      <c r="AU2" s="12">
+        <f t="shared" si="0"/>
+        <v>300</v>
+      </c>
+      <c r="AV2" s="12">
+        <f t="shared" si="0"/>
+        <v>300</v>
+      </c>
+      <c r="AW2" s="12">
+        <f t="shared" si="0"/>
+        <v>300</v>
+      </c>
+      <c r="AX2" s="12">
+        <f t="shared" si="0"/>
+        <v>300</v>
+      </c>
+      <c r="AY2" s="12">
+        <f t="shared" si="0"/>
+        <v>300</v>
+      </c>
+      <c r="AZ2" s="12">
+        <f t="shared" si="0"/>
+        <v>300</v>
+      </c>
+      <c r="BA2" s="12">
+        <f t="shared" si="0"/>
+        <v>300</v>
+      </c>
+      <c r="BB2" s="12">
+        <f t="shared" si="0"/>
+        <v>300</v>
+      </c>
+      <c r="BC2" s="12">
         <f t="shared" si="0"/>
         <v>300</v>
       </c>
@@ -4028,21 +5026,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement/>
-</p:properties>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101009A9DAB439B36DB4795F39C4E722C7BC4" ma:contentTypeVersion="4" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="44674c89fa9bc5e97a878a6680c46188">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="79748b23-d81a-423e-9112-21109dc864e6" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="447839a363ea5a12024b5bf1ab53ed90" ns2:_="">
     <xsd:import namespace="79748b23-d81a-423e-9112-21109dc864e6"/>
@@ -4186,14 +5169,52 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement/>
+</p:properties>
+</file>
+
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{150680C4-F692-4EAD-A60B-637CE72108F8}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9112A27B-23A8-4AD5-88DA-C23BF7A8AF48}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="79748b23-d81a-423e-9112-21109dc864e6"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{534D3644-ED23-42A8-AF43-0EB127BD4A83}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{534D3644-ED23-42A8-AF43-0EB127BD4A83}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9112A27B-23A8-4AD5-88DA-C23BF7A8AF48}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{150680C4-F692-4EAD-A60B-637CE72108F8}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>